<commit_message>
Half Day Logic woking
</commit_message>
<xml_diff>
--- a/notification_configs/02_manager_summary_notifications.xlsx
+++ b/notification_configs/02_manager_summary_notifications.xlsx
@@ -702,20 +702,20 @@
         </is>
       </c>
       <c r="U2" t="n">
+        <v>2</v>
+      </c>
+      <c r="V2" t="n">
         <v>1</v>
-      </c>
-      <c r="V2" t="n">
-        <v>2</v>
       </c>
       <c r="W2" t="n">
         <v>1</v>
       </c>
       <c r="X2" t="n">
-        <v>33.3</v>
+        <v>66.7</v>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>2025-09-10 21:39:55</t>
+          <t>2025-09-10 22:25:58</t>
         </is>
       </c>
     </row>

</xml_diff>